<commit_message>
* chore: Add object type column to objects sheet in script
</commit_message>
<xml_diff>
--- a/Dokumentace/Scénář.xlsx
+++ b/Dokumentace/Scénář.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Chipotle\Columbo\Dokumentace\Nový scénář\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lukas\source\repos\Definitive Chipotle\Dokumentace\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D709EA63-0C9B-4595-BC6D-70181571D669}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD80A7DC-01C9-40B2-8E90-F1F86E9D14E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="0" showVerticalScroll="0" showSheetTabs="0" xWindow="0" yWindow="0" windowWidth="2370" windowHeight="560" activeTab="6" xr2:uid="{F3D84F34-5C87-417A-B7B4-147627C7DFDB}"/>
+    <workbookView showHorizontalScroll="0" showVerticalScroll="0" showSheetTabs="0" xWindow="0" yWindow="0" windowWidth="2370" windowHeight="560" activeTab="7" xr2:uid="{F3D84F34-5C87-417A-B7B4-147627C7DFDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Graf1" sheetId="7" r:id="rId1"/>
@@ -31,7 +31,6 @@
     <definedName name="TitleRegion5..I300">Objekty!$A$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -49,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1990" uniqueCount="1053">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1991" uniqueCount="1053">
   <si>
     <t>ID</t>
   </si>
@@ -9708,13 +9707,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB182C5E-7FDA-4783-BD11-42549E8A6D11}">
-  <dimension ref="A1:F237"/>
+  <dimension ref="A1:G237"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="6" width="8.7265625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
@@ -9733,8 +9732,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G1" s="15" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -9750,7 +9752,7 @@
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
     </row>
-    <row r="3" spans="1:6" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -9766,7 +9768,7 @@
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
     </row>
-    <row r="4" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
@@ -9782,7 +9784,7 @@
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
     </row>
-    <row r="5" spans="1:6" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" ht="131" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -9798,7 +9800,7 @@
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
     </row>
-    <row r="6" spans="1:6" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" ht="131" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -9814,7 +9816,7 @@
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
     </row>
-    <row r="7" spans="1:6" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="131" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>22</v>
       </c>
@@ -9830,7 +9832,7 @@
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
     </row>
-    <row r="8" spans="1:6" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>25</v>
       </c>
@@ -9846,7 +9848,7 @@
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
     </row>
-    <row r="9" spans="1:6" ht="189" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" ht="189" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>28</v>
       </c>
@@ -9862,7 +9864,7 @@
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
     </row>
-    <row r="10" spans="1:6" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" ht="131" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>31</v>
       </c>
@@ -9878,7 +9880,7 @@
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
     </row>
-    <row r="11" spans="1:6" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" ht="73" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>34</v>
       </c>
@@ -9894,7 +9896,7 @@
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
     </row>
-    <row r="12" spans="1:6" ht="247" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" ht="247" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>37</v>
       </c>
@@ -9910,7 +9912,7 @@
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
     </row>
-    <row r="13" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>40</v>
       </c>
@@ -9926,7 +9928,7 @@
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
     </row>
-    <row r="14" spans="1:6" ht="174.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" ht="174.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>43</v>
       </c>
@@ -9942,7 +9944,7 @@
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
     </row>
-    <row r="15" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>46</v>
       </c>
@@ -9958,7 +9960,7 @@
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
     </row>
-    <row r="16" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>50</v>
       </c>

</xml_diff>

<commit_message>
* chore: little changes in the script
</commit_message>
<xml_diff>
--- a/Dokumentace/Scénář.xlsx
+++ b/Dokumentace/Scénář.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Chipotle\Columbo\Dokumentace\Nový scénář\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lukas\source\repos\Definitive Chipotle\Dokumentace\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D709EA63-0C9B-4595-BC6D-70181571D669}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD80A7DC-01C9-40B2-8E90-F1F86E9D14E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="0" showVerticalScroll="0" showSheetTabs="0" xWindow="0" yWindow="0" windowWidth="2370" windowHeight="560" activeTab="6" xr2:uid="{F3D84F34-5C87-417A-B7B4-147627C7DFDB}"/>
+    <workbookView showHorizontalScroll="0" showVerticalScroll="0" showSheetTabs="0" xWindow="0" yWindow="0" windowWidth="2370" windowHeight="560" activeTab="7" xr2:uid="{F3D84F34-5C87-417A-B7B4-147627C7DFDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Graf1" sheetId="7" r:id="rId1"/>
@@ -31,7 +31,6 @@
     <definedName name="TitleRegion5..I300">Objekty!$A$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -49,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1990" uniqueCount="1053">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1991" uniqueCount="1053">
   <si>
     <t>ID</t>
   </si>
@@ -9708,13 +9707,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB182C5E-7FDA-4783-BD11-42549E8A6D11}">
-  <dimension ref="A1:F237"/>
+  <dimension ref="A1:G237"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="6" width="8.7265625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
@@ -9733,8 +9732,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="G1" s="15" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -9750,7 +9752,7 @@
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
     </row>
-    <row r="3" spans="1:6" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -9766,7 +9768,7 @@
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
     </row>
-    <row r="4" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
@@ -9782,7 +9784,7 @@
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
     </row>
-    <row r="5" spans="1:6" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" ht="131" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -9798,7 +9800,7 @@
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
     </row>
-    <row r="6" spans="1:6" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" ht="131" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -9814,7 +9816,7 @@
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
     </row>
-    <row r="7" spans="1:6" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="131" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>22</v>
       </c>
@@ -9830,7 +9832,7 @@
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
     </row>
-    <row r="8" spans="1:6" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>25</v>
       </c>
@@ -9846,7 +9848,7 @@
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
     </row>
-    <row r="9" spans="1:6" ht="189" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" ht="189" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>28</v>
       </c>
@@ -9862,7 +9864,7 @@
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
     </row>
-    <row r="10" spans="1:6" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" ht="131" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>31</v>
       </c>
@@ -9878,7 +9880,7 @@
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
     </row>
-    <row r="11" spans="1:6" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" ht="73" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>34</v>
       </c>
@@ -9894,7 +9896,7 @@
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
     </row>
-    <row r="12" spans="1:6" ht="247" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" ht="247" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>37</v>
       </c>
@@ -9910,7 +9912,7 @@
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
     </row>
-    <row r="13" spans="1:6" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>40</v>
       </c>
@@ -9926,7 +9928,7 @@
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
     </row>
-    <row r="14" spans="1:6" ht="174.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" ht="174.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>43</v>
       </c>
@@ -9942,7 +9944,7 @@
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
     </row>
-    <row r="15" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>46</v>
       </c>
@@ -9958,7 +9960,7 @@
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
     </row>
-    <row r="16" spans="1:6" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>50</v>
       </c>

</xml_diff>